<commit_message>
auto: session 2026-10-29 10:58
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11-bao-gia-khach/Bao-Gia-PR-Bao-Link-Dofollow-EPC-Hannah-2026-10-29.xlsx
+++ b/11-bao-gia-khach/Bao-Gia-PR-Bao-Link-Dofollow-EPC-Hannah-2026-10-29.xlsx
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -576,7 +576,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BÁO GIÁ BOOKING BÁO PR - BÁO CÓ LINK DOFOLLOW VÀ BÁO NGÀNH</t>
+          <t>BÁO GIÁ BOOKING BÁO PR - BÁO CÓ LINK DOFOLLOW, BÁO NGÀNH VÀ BÁO LỚN TOÀN QUỐC</t>
         </is>
       </c>
     </row>
@@ -935,83 +935,83 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
+          <t>Doanhnghiepvn.vn</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Mục phù hợp, bài lấy link</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 3 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Dofollow</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>4260000</v>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>26%</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>3150000</v>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>3402000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
           <t>Vietnambiz.vn</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Mục Góc doanh nghiệp, kèm 1 link dofollow</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>1.000 từ, 3 ảnh, 1 link</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>Dofollow</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n">
-        <v>6100000</v>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>26%</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="n">
+      <c r="F17" s="10" t="n">
+        <v>6020000</v>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="n">
         <v>4510000</v>
       </c>
-      <c r="I16" s="12" t="n">
+      <c r="I17" s="12" t="n">
         <v>4870800</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>BÁO NGÀNH CÔNG THƯƠNG, ĐẦU TƯ, XÂY DỰNG</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Congthuong.vn</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Mục phù hợp</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Dưới 700 từ, 3 ảnh, 1 link</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>Toà soạn duyệt loại link</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>10670000</v>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="I18" s="12" t="n">
-        <v>8640000</v>
       </c>
     </row>
     <row r="19">
@@ -1020,26 +1020,26 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Baodautu.vn</t>
+          <t>Congthuong.vn</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Thông tin doanh nghiệp</t>
+          <t>Mục phù hợp</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>1.000 từ, 3 ảnh, không link</t>
+          <t>Dưới 700 từ, 3 ảnh, 1 link</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Không gắn link (mua thêm bên dưới)</t>
+          <t>Toà soạn duyệt loại link</t>
         </is>
       </c>
       <c r="F19" s="10" t="n">
-        <v>5420000</v>
+        <v>11120000</v>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
@@ -1047,10 +1047,10 @@
         </is>
       </c>
       <c r="H19" s="11" t="n">
-        <v>3900000</v>
+        <v>8000000</v>
       </c>
       <c r="I19" s="12" t="n">
-        <v>4212000</v>
+        <v>8640000</v>
       </c>
     </row>
     <row r="20">
@@ -1059,12 +1059,12 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Vietnambiz.vn</t>
+          <t>Baodautu.vn</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Mục phù hợp</t>
+          <t>Thông tin doanh nghiệp</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="F20" s="10" t="n">
-        <v>3060000</v>
+        <v>5420000</v>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
@@ -1086,10 +1086,10 @@
         </is>
       </c>
       <c r="H20" s="11" t="n">
-        <v>2200000</v>
+        <v>3900000</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>2376000</v>
+        <v>4212000</v>
       </c>
     </row>
     <row r="21">
@@ -1098,77 +1098,83 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
+          <t>Vietnambiz.vn</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Mục phù hợp</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 3 ảnh, không link</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Không gắn link (mua thêm bên dưới)</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="n">
+        <v>3020000</v>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>2376000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
           <t>Baoxaydung.vn</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Mục phù hợp</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>1.000 từ, 3 ảnh, không link</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>Không gắn link (mua thêm bên dưới)</t>
         </is>
       </c>
-      <c r="F21" s="10" t="n">
-        <v>2610000</v>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>27%</t>
-        </is>
-      </c>
-      <c r="H21" s="11" t="n">
+      <c r="F22" s="10" t="n">
+        <v>2440000</v>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="n">
         <v>1900000</v>
       </c>
-      <c r="I21" s="12" t="n">
+      <c r="I22" s="12" t="n">
         <v>2052000</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>DỊCH VỤ CỘNG THÊM (CHÈN THÊM LINK VÀO BÀI ĐÃ ĐẶT)</t>
-        </is>
-      </c>
-    </row>
     <row r="23">
-      <c r="A23" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Baodautu.vn</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Chèn thêm 1 link</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Cộng thêm vào bài đã đặt trên cùng báo</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Nofollow</t>
-        </is>
-      </c>
-      <c r="F23" s="13" t="n"/>
-      <c r="G23" s="8" t="inlineStr"/>
-      <c r="H23" s="11" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="I23" s="12" t="n">
-        <v>1080000</v>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>BÁO LỚN TOÀN QUỐC (LINK NOFOLLOW, TĂNG NHẬN DIỆN)</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1177,17 +1183,17 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Vietnambiz.vn</t>
+          <t>Vnexpress.net</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Chèn thêm 1 link</t>
+          <t>Tiểu mục Doanh nghiệp viết, lên Box Thông tin doanh nghiệp trang chủ, duy trì 6 tháng</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Cộng thêm vào bài đã đặt trên cùng báo</t>
+          <t>1.000 từ, 3 ảnh, 2 link</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -1195,13 +1201,19 @@
           <t>Nofollow</t>
         </is>
       </c>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="8" t="inlineStr"/>
+      <c r="F24" s="10" t="n">
+        <v>10130000</v>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>23%</t>
+        </is>
+      </c>
       <c r="H24" s="11" t="n">
-        <v>550000</v>
+        <v>7800000</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>594000</v>
+        <v>8424000</v>
       </c>
     </row>
     <row r="25">
@@ -1210,106 +1222,948 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
+          <t>Vnexpress.net</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Tiểu mục Doanh nghiệp viết, lên Box Thông tin doanh nghiệp trang chủ, duy trì 2 năm</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 3 ảnh, 2 link</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>14940000</v>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>21%</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="n">
+        <v>11800000</v>
+      </c>
+      <c r="I25" s="12" t="n">
+        <v>12744000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Vnexpress.net</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Tiểu mục Doanh nghiệp viết, lên Box Thông tin doanh nghiệp trang chủ, không giới hạn thời gian</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 3 ảnh, 2 link</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>20680000</v>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>26%</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="n">
+        <v>15300000</v>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>16524000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Vnexpress.net</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Tiểu mục NetZero (Kinh doanh), top 4 trở xuống</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 3 ảnh, 2 link</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>20860000</v>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>23%</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="n">
+        <v>16060000</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>17344800</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Thanhnien.vn</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Box Bạn cần biết ngoài trang chủ</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>800 từ, 4 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>9120000</v>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>24%</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="n">
+        <v>6930000</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>7484400</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Thanhnien.vn</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Tin ngắn mục Bạn cần biết (tiểu mục Kinh tế)</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>300 từ, 1 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="n">
+        <v>4760000</v>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="n">
+        <v>3470000</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>3747600</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Thanhnien.vn</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Tiểu mục phù hợp thuộc Kinh tế hoặc Công nghệ</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Dưới 1.000 từ, 5 ảnh, 2 link</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>16660000</v>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="n">
+        <v>12990000</v>
+      </c>
+      <c r="I30" s="12" t="n">
+        <v>14029200</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Dantri.com.vn</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Tiểu mục thuộc Kinh doanh hoặc Đời sống</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 5 ảnh, link tĩnh (mua thêm link bên dưới)</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="n">
+        <v>14590000</v>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="n">
+        <v>10500000</v>
+      </c>
+      <c r="I31" s="12" t="n">
+        <v>11340000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Vietnamnet.vn</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Tiểu mục Kinh doanh, top 6 trở xuống</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 5 ảnh, link tĩnh (mua thêm link bên dưới)</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="n">
+        <v>6270000</v>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>21%</t>
+        </is>
+      </c>
+      <c r="H32" s="11" t="n">
+        <v>4950000</v>
+      </c>
+      <c r="I32" s="12" t="n">
+        <v>5346000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Tienphong.vn</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Chuyên mục Kinh tế hoặc Khoa học</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Dưới 800 từ, 2 ảnh, 1 link tên miền .vn</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="n">
+        <v>5790000</v>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>24%</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="n">
+        <v>4400000</v>
+      </c>
+      <c r="I33" s="12" t="n">
+        <v>4752000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>24h.com.vn</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Bài PR loại 2 mục Kinh doanh hoặc Thị trường tiêu dùng (Box Tin tức thị trường)</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 5 ảnh, 3 link</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="n">
+        <v>6170000</v>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="I34" s="12" t="n">
+        <v>4860000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Cafef.vn</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Box Thông cáo báo chí trên trang chủ 1 ngày</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 5 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="n">
+        <v>6930000</v>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="H35" s="11" t="n">
+        <v>5400000</v>
+      </c>
+      <c r="I35" s="12" t="n">
+        <v>5832000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Cafef.vn</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Box Tin doanh nghiệp trên trang chủ 1 ngày</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 5 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>8920000</v>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>26%</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="n">
+        <v>6600000</v>
+      </c>
+      <c r="I36" s="12" t="n">
+        <v>7128000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Cafef.vn</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Chuyên mục phù hợp, trôi dần theo thời gian</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>1.500 từ, 5 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>11860000</v>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>23%</t>
+        </is>
+      </c>
+      <c r="H37" s="11" t="n">
+        <v>9130000</v>
+      </c>
+      <c r="I37" s="12" t="n">
+        <v>9860400</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Cafebiz.vn</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Bài thứ 6 Stream 1 trang chủ, lưu mục phù hợp</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>1.500 từ, 5 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>13960000</v>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="n">
+        <v>10050000</v>
+      </c>
+      <c r="I38" s="12" t="n">
+        <v>10854000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Cafebiz.vn</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Bài thứ 6 Stream 2 trang chủ 2 giờ, lưu mục phù hợp</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>1.500 từ, 5 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>9620000</v>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>24%</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="n">
+        <v>7310000</v>
+      </c>
+      <c r="I39" s="12" t="n">
+        <v>7894800</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Cafebiz.vn</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Chuyên mục phù hợp</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 3 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="n">
+        <v>6090000</v>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>26%</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="I40" s="12" t="n">
+        <v>4860000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Vneconomy.vn</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Mục phù hợp</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Dưới 1.000 từ, 3 ảnh, không link</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="n">
+        <v>9500000</v>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>21%</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="I41" s="12" t="n">
+        <v>8100000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Nguoiquansat.vn</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Chuyên mục, bài lấy link</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>1.000 từ, 5 ảnh, 1 link</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="n">
+        <v>3850000</v>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="n">
+        <v>2810000</v>
+      </c>
+      <c r="I42" s="12" t="n">
+        <v>3034800</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>DỊCH VỤ CỘNG THÊM (CHÈN THÊM LINK VÀO BÀI ĐÃ ĐẶT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Baodautu.vn</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Chèn thêm 1 link</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Cộng thêm vào bài đã đặt trên cùng báo</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="n"/>
+      <c r="G44" s="8" t="inlineStr"/>
+      <c r="H44" s="11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I44" s="12" t="n">
+        <v>1080000</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Vietnambiz.vn</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Chèn thêm 1 link</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Cộng thêm vào bài đã đặt trên cùng báo</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F45" s="13" t="n"/>
+      <c r="G45" s="8" t="inlineStr"/>
+      <c r="H45" s="11" t="n">
+        <v>550000</v>
+      </c>
+      <c r="I45" s="12" t="n">
+        <v>594000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
           <t>Baoxaydung.vn</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C46" s="9" t="inlineStr">
         <is>
           <t>Chèn thêm 1 link</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D46" s="9" t="inlineStr">
         <is>
           <t>Cộng thêm vào bài đã đặt trên cùng báo</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E46" s="9" t="inlineStr">
         <is>
           <t>Nofollow</t>
         </is>
       </c>
-      <c r="F25" s="13" t="n"/>
-      <c r="G25" s="8" t="inlineStr"/>
-      <c r="H25" s="11" t="n">
+      <c r="F46" s="13" t="n"/>
+      <c r="G46" s="8" t="inlineStr"/>
+      <c r="H46" s="11" t="n">
         <v>1100000</v>
       </c>
-      <c r="I25" s="12" t="n">
+      <c r="I46" s="12" t="n">
         <v>1188000</v>
       </c>
     </row>
-    <row r="26">
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Dantri.com.vn</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Chèn thêm 1 link</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Cộng thêm vào bài đã đặt trên cùng báo</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F47" s="13" t="n"/>
+      <c r="G47" s="8" t="inlineStr"/>
+      <c r="H47" s="11" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I47" s="12" t="n">
+        <v>540000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Vietnamnet.vn</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Chèn thêm 1 link, hiển thị 3 tháng</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>Cộng thêm vào bài đã đặt trên cùng báo</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>Nofollow</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="n"/>
+      <c r="G48" s="8" t="inlineStr"/>
+      <c r="H48" s="11" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="I48" s="12" t="n">
+        <v>5400000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" s="5" t="n"/>
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="5" t="n"/>
+      <c r="H49" s="5" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
         <is>
           <t>GHI CHÚ</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="51" ht="34" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>- Giá tính cho 01 bài (hoặc 01 link với dịch vụ cộng thêm), chưa gồm VAT 8%. Cột cuối đã cộng VAT 8% để Quý khách tiện đối chiếu.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="34" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="52" ht="34" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>- Nội dung bài: Quý khách cung cấp thông tin, DigicomVN biên tập bài PR theo quy cách từng báo và gửi Quý khách duyệt trước khi gửi toà soạn - không tính phí viết bài.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="34" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>- Loại link: các báo trong nhóm "Báo có link dofollow" gắn link dofollow trỏ về website của Quý khách. Báo ngành (Công Thương, Đầu tư, Xây dựng, Vietnambiz mục thường) gắn link nofollow hoặc theo duyệt của toà soạn.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="34" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>- Gợi ý: nếu ưu tiên link dofollow, 6 báo đầu tiên (Diễn đàn Doanh nghiệp, Tạp chí Xây dựng, Báo Cà Mau, Báo Cần Thơ, Báo Lâm Đồng, Báo Quảng Ninh) đều có link dofollow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="34" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>- Thời gian tồn tại: bài lưu trên báo không giới hạn thời gian.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="34" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="53" ht="34" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>- Loại link: các báo trong nhóm "Báo có link dofollow" gắn link dofollow trỏ về website của Quý khách. Báo ngành (Công Thương, Đầu tư, Xây dựng, Vietnambiz mục thường) và báo lớn toàn quốc (VnExpress, Thanh Niên, Dân Trí, VietNamNet, CafeF...) gắn link nofollow hoặc theo duyệt của toà soạn; nhóm báo lớn phù hợp mục tiêu tăng nhận diện và độ tin cậy thương hiệu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="34" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>- Gợi ý: nếu ưu tiên link dofollow, chọn trong nhóm "Báo có link dofollow" (Diễn đàn Doanh nghiệp, Tạp chí Xây dựng, Báo Cà Mau, Báo Cần Thơ, Báo Lâm Đồng, Báo Quảng Ninh, Doanh nghiệp Việt Nam, Vietnambiz).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="34" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>- Thời gian tồn tại: bài lưu trên báo không giới hạn thời gian, trừ các vị trí ghi rõ thời hạn (VnExpress 6 tháng/2 năm, link chèn thêm VietNamNet 3 tháng).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="34" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>- Nhãn bài: tuỳ vị trí, toà soạn có thể gắn nhãn thông tin doanh nghiệp theo quy định của từng báo. Toà soạn có thể biên tập lại câu chữ; lịch đăng và chuyên mục cuối cùng do toà soạn duyệt.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="A29:I29"/>
+  <mergeCells count="17">
+    <mergeCell ref="A52:I52"/>
+    <mergeCell ref="A43:I43"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A33:I33"/>
-    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="A32:I32"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A23:I23"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B5:I5"/>
     <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A27:I27"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="A55:I55"/>
+    <mergeCell ref="A50:I50"/>
     <mergeCell ref="B4:I4"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>